<commit_message>
Fix syntax error around catch block in peso-talla.js restoring main options loop structure
</commit_message>
<xml_diff>
--- a/docs/f4.m3.pp_formato_cambio_datos_basicos_personas_v5.xlsx
+++ b/docs/f4.m3.pp_formato_cambio_datos_basicos_personas_v5.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="79">
   <si>
     <t xml:space="preserve">PROCESO
 PROMOCIÓN Y PREVENCIÓN
@@ -149,6 +149,9 @@
   </si>
   <si>
     <t>TIPO DE DOCUMENTO MAL DIGITADO - FECHA DE NACIMIENTO MAL DIGITADA - SEXO MAL DIGITADO</t>
+  </si>
+  <si>
+    <t>Error en Diligenciamiento de Datos Basicos</t>
   </si>
   <si>
     <t>BOLIVAR</t>
@@ -1873,32 +1876,80 @@
     <row r="7" ht="15.75" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="35"/>
       <c r="B7" s="36"/>
-      <c r="C7" s="48"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="38"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
-      <c r="I7" s="49"/>
-      <c r="J7" s="40"/>
-      <c r="K7" s="49"/>
-      <c r="L7" s="51"/>
-      <c r="M7" s="36"/>
-      <c r="N7" s="48"/>
-      <c r="O7" s="38"/>
-      <c r="P7" s="38"/>
-      <c r="Q7" s="49"/>
-      <c r="R7" s="49"/>
-      <c r="S7" s="50"/>
-      <c r="T7" s="49"/>
-      <c r="U7" s="40"/>
-      <c r="V7" s="49"/>
-      <c r="W7" s="51"/>
-      <c r="X7" s="42"/>
-      <c r="Y7" s="43"/>
+      <c r="C7" s="48" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="49" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="50" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="J7" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="L7" s="51" t="s">
+        <v>38</v>
+      </c>
+      <c r="M7" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="N7" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="O7" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="P7" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q7" s="49" t="s">
+        <v>32</v>
+      </c>
+      <c r="R7" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="S7" s="50" t="s">
+        <v>34</v>
+      </c>
+      <c r="T7" s="49" t="s">
+        <v>38</v>
+      </c>
+      <c r="U7" s="40" t="s">
+        <v>38</v>
+      </c>
+      <c r="V7" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="W7" s="51" t="s">
+        <v>38</v>
+      </c>
+      <c r="X7" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y7" s="43" t="s">
+        <v>42</v>
+      </c>
       <c r="Z7" s="52"/>
       <c r="AA7" s="53"/>
-      <c r="AB7" s="54"/>
+      <c r="AB7" s="54" t="s">
+        <v>41</v>
+      </c>
       <c r="AC7" s="55"/>
       <c r="AD7" s="56"/>
       <c r="AG7" s="47"/>
@@ -2034,7 +2085,7 @@
       <c r="AC11" s="55"/>
       <c r="AD11" s="56"/>
       <c r="AG11" s="47" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2069,7 +2120,7 @@
       <c r="AC12" s="55"/>
       <c r="AD12" s="56"/>
       <c r="AG12" s="47" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2104,7 +2155,7 @@
       <c r="AC13" s="55"/>
       <c r="AD13" s="56"/>
       <c r="AG13" s="47" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2139,7 +2190,7 @@
       <c r="AC14" s="55"/>
       <c r="AD14" s="56"/>
       <c r="AG14" s="47" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2174,7 +2225,7 @@
       <c r="AC15" s="55"/>
       <c r="AD15" s="56"/>
       <c r="AG15" s="47" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2209,7 +2260,7 @@
       <c r="AC16" s="55"/>
       <c r="AD16" s="56"/>
       <c r="AG16" s="47" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2244,7 +2295,7 @@
       <c r="AC17" s="55"/>
       <c r="AD17" s="56"/>
       <c r="AG17" s="47" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2279,7 +2330,7 @@
       <c r="AC18" s="55"/>
       <c r="AD18" s="56"/>
       <c r="AG18" s="47" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2314,7 +2365,7 @@
       <c r="AC19" s="55"/>
       <c r="AD19" s="56"/>
       <c r="AG19" s="47" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2349,17 +2400,17 @@
       <c r="AC20" s="66"/>
       <c r="AD20" s="67"/>
       <c r="AG20" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="33:33" x14ac:dyDescent="0.25">
       <c r="AG21" s="47" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" ht="16.9" customHeight="1" spans="1:30" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="69" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B22" s="69"/>
       <c r="C22" s="69"/>
@@ -2393,7 +2444,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:30" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="70" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B23" s="70"/>
       <c r="C23" s="70"/>
@@ -2427,7 +2478,7 @@
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:30" s="68" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="70" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B24" s="70"/>
       <c r="C24" s="70"/>
@@ -2554,167 +2605,167 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="71" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="71" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="71" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="71" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="71" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="71" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="71" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="71" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="71" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="71" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="71" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="71" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="71" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="71" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="71" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="71" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="71" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="71" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="71" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="71" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="71" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="71" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="71" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="71" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="71" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="71" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="71" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="71" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="71" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="71" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="71" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Script 12 draft saving by sanitizing Gmail passwords, adding local .eml fallback, and preventing script crashes
</commit_message>
<xml_diff>
--- a/docs/f4.m3.pp_formato_cambio_datos_basicos_personas_v5.xlsx
+++ b/docs/f4.m3.pp_formato_cambio_datos_basicos_personas_v5.xlsx
@@ -151,7 +151,7 @@
     <t>Error en Diligenciamiento de Datos Basicos</t>
   </si>
   <si>
-    <t>TIPO DE DOCUMENTO MAL DIGITADO - FECHA DE NACIMIENTO MAL DIGITADA - SEXO MAL DIGITADO - MUNICIPIO DE NACIMIENTO MAL DIGITADO</t>
+    <t>CAMBIAR DE (TI) A (CC)</t>
   </si>
   <si>
     <t>BOLIVAR</t>
@@ -1841,7 +1841,7 @@
         <v>40</v>
       </c>
       <c r="U6" s="40" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="V6" s="40" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Fix Option 12 Observacion column placement to Column 27 (AA) under the orange Observacion header
</commit_message>
<xml_diff>
--- a/docs/f4.m3.pp_formato_cambio_datos_basicos_personas_v5.xlsx
+++ b/docs/f4.m3.pp_formato_cambio_datos_basicos_personas_v5.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="77">
   <si>
     <t xml:space="preserve">PROCESO
 PROMOCIÓN Y PREVENCIÓN
@@ -133,7 +133,7 @@
     <t>02/11/2007</t>
   </si>
   <si>
-    <t>MUJER</t>
+    <t>FEMENINO</t>
   </si>
   <si>
     <t>COLOMBIA</t>
@@ -146,6 +146,9 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>BOGOTA, D.C.</t>
   </si>
   <si>
     <t>Error en Diligenciamiento de Datos Basicos</t>
@@ -1785,80 +1788,80 @@
     </row>
     <row r="6" ht="15.75" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="35"/>
-      <c r="B6" s="36"/>
+      <c r="B6" s="36" t="s">
+        <v>29</v>
+      </c>
       <c r="C6" s="37" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E6" s="38" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F6" s="38" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H6" s="39" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="40" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J6" s="40" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K6" s="40" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="L6" s="41" t="s">
         <v>38</v>
       </c>
       <c r="M6" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="O6" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="P6" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q6" s="38" t="s">
+        <v>33</v>
+      </c>
+      <c r="R6" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="S6" s="39" t="s">
+        <v>40</v>
+      </c>
+      <c r="T6" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="U6" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="V6" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="N6" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="O6" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="P6" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q6" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="R6" s="38" t="s">
-        <v>33</v>
-      </c>
-      <c r="S6" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="T6" s="40" t="s">
-        <v>40</v>
-      </c>
-      <c r="U6" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="V6" s="40" t="s">
-        <v>37</v>
-      </c>
       <c r="W6" s="41" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="X6" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y6" s="43" t="s">
-        <v>41</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="Y6" s="43"/>
       <c r="Z6" s="44"/>
       <c r="AA6" s="42"/>
       <c r="AB6" s="45" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="AC6" s="43"/>
       <c r="AD6" s="46"/>
@@ -2028,7 +2031,7 @@
       <c r="AC11" s="55"/>
       <c r="AD11" s="56"/>
       <c r="AG11" s="47" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2063,7 +2066,7 @@
       <c r="AC12" s="55"/>
       <c r="AD12" s="56"/>
       <c r="AG12" s="47" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2098,7 +2101,7 @@
       <c r="AC13" s="55"/>
       <c r="AD13" s="56"/>
       <c r="AG13" s="47" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2133,7 +2136,7 @@
       <c r="AC14" s="55"/>
       <c r="AD14" s="56"/>
       <c r="AG14" s="47" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2168,7 +2171,7 @@
       <c r="AC15" s="55"/>
       <c r="AD15" s="56"/>
       <c r="AG15" s="47" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2203,7 +2206,7 @@
       <c r="AC16" s="55"/>
       <c r="AD16" s="56"/>
       <c r="AG16" s="47" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2238,7 +2241,7 @@
       <c r="AC17" s="55"/>
       <c r="AD17" s="56"/>
       <c r="AG17" s="47" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2273,7 +2276,7 @@
       <c r="AC18" s="55"/>
       <c r="AD18" s="56"/>
       <c r="AG18" s="47" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2308,7 +2311,7 @@
       <c r="AC19" s="55"/>
       <c r="AD19" s="56"/>
       <c r="AG19" s="47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -2343,7 +2346,7 @@
       <c r="AC20" s="66"/>
       <c r="AD20" s="67"/>
       <c r="AG20" s="47" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.25">
@@ -2378,7 +2381,7 @@
       <c r="AC21" s="1"/>
       <c r="AD21" s="1"/>
       <c r="AG21" s="47" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" ht="16.9" customHeight="1" spans="1:30" s="68" customFormat="1" x14ac:dyDescent="0.25">
@@ -5004,167 +5007,167 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="71" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="71" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="71" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="71" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="71" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="71" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="71" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="71" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="71" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="71" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="71" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="71" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="71" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="71" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="71" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="71" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="71" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="71" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="71" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="71" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="71" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="71" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="71" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="71" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="71" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="71" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="71" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="71" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="71" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="71" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="71" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>